<commit_message>
Add pivot table summarizing sales amount by ship mode and month
- Rows: Month
- Columns: Ship Mode
- Values: Sum of Sales Amount
- Built on top of the cleaned/combined dataset from Power Query steps
</commit_message>
<xml_diff>
--- a/Excel Automation Combine Multiple Files Using Power Query/Consolidated Files With Power Query.xlsx
+++ b/Excel Automation Combine Multiple Files Using Power Query/Consolidated Files With Power Query.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerwi\OneDrive\Desktop\August\Github Repo\power-query-data-cleaning-automation\Excel Automation Combine Multiple Files Using Power Query\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38883C7D-9324-4449-92A4-4539F0405196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E253DFA-6E3D-4AB1-9F05-600D49FF10D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B69BFFAD-2A01-46BE-89B6-740D3216DF36}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   <definedNames>
     <definedName name="ExternalData_1" localSheetId="0" hidden="1">'Consolidated File'!$A$1:$M$901</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <pivotCaches>
     <pivotCache cacheId="4" r:id="rId3"/>
   </pivotCaches>
@@ -892,6 +892,1238 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[Consolidated Files With Power Query.xlsx]Report!PivotTable1</c:name>
+    <c:fmtId val="0"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Report!$B$4:$B$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Express</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Report!$A$6:$A$12</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Jan</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Report!$B$6:$B$12</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>3041955</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3186100</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3058893</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3071730</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2924927</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2514552</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-6053-4871-9F5F-F8577DBEBE10}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Report!$C$4:$C$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Same Day</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Report!$A$6:$A$12</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Jan</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Report!$C$6:$C$12</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>2337403</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3309662</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2248949</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3204264</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2853396</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2581130</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-6053-4871-9F5F-F8577DBEBE10}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Report!$D$4:$D$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Standard</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Report!$A$6:$A$12</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Jan</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Report!$D$6:$D$12</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>3182183</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1762064</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2423727</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2281188</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2781304</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2583429</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-6053-4871-9F5F-F8577DBEBE10}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1994928383"/>
+        <c:axId val="1994928863"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1994928383"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1994928863"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1994928863"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="#,##0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1994928383"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>109537</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>185737</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C72EA050-B8A0-F82D-3372-DF74531D1594}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Asus" refreshedDate="46223.665681481485" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="900" xr:uid="{2799B9B7-3019-4065-805D-50E3D7947C09}">
   <cacheSource type="worksheet">
@@ -15033,7 +16265,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FA09C0C6-D2A2-483C-975A-3DD3727DF74B}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FA09C0C6-D2A2-483C-975A-3DD3727DF74B}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A4:E12" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="15">
     <pivotField showAll="0"/>
@@ -15697,6 +16929,44 @@
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
+  <chartFormats count="3">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="3" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="3" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="3" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -53194,6 +54464,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add chart visualizing sales amount by month and ship mode
</commit_message>
<xml_diff>
--- a/Excel Automation Combine Multiple Files Using Power Query/Consolidated Files With Power Query.xlsx
+++ b/Excel Automation Combine Multiple Files Using Power Query/Consolidated Files With Power Query.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerwi\OneDrive\Desktop\August\Github Repo\power-query-data-cleaning-automation\Excel Automation Combine Multiple Files Using Power Query\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E253DFA-6E3D-4AB1-9F05-600D49FF10D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FFB0910-357A-4C06-97CA-3DA6F36EBDFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B69BFFAD-2A01-46BE-89B6-740D3216DF36}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6327" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6328" uniqueCount="88">
   <si>
     <t>Order ID</t>
   </si>
@@ -308,6 +308,9 @@
   </si>
   <si>
     <t>Sum of Sales Amount</t>
+  </si>
+  <si>
+    <t>s</t>
   </si>
 </sst>
 </file>
@@ -54309,7 +54312,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{222C8973-2D6F-4025-A0C3-8463CBA55F3C}">
-  <dimension ref="A4:E12"/>
+  <dimension ref="A4:J14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.28515625" bestFit="1" customWidth="1"/>
@@ -54318,7 +54321,7 @@
     <col min="5" max="5" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>86</v>
       </c>
@@ -54326,7 +54329,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>79</v>
       </c>
@@ -54343,7 +54346,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>80</v>
       </c>
@@ -54360,7 +54363,7 @@
         <v>8561541</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>81</v>
       </c>
@@ -54377,7 +54380,7 @@
         <v>8257826</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>82</v>
       </c>
@@ -54394,7 +54397,7 @@
         <v>7731569</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>83</v>
       </c>
@@ -54411,7 +54414,7 @@
         <v>8557182</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>84</v>
       </c>
@@ -54428,7 +54431,7 @@
         <v>8559627</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>85</v>
       </c>
@@ -54445,7 +54448,7 @@
         <v>7679111</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>78</v>
       </c>
@@ -54460,6 +54463,11 @@
       </c>
       <c r="E12" s="5">
         <v>49346856</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J14" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>